<commit_message>
refactor: rename user table, add check constraints, and create triggers in data dictionary
</commit_message>
<xml_diff>
--- a/SysCall-BackEnd/Dicionario de Dados/Dicionario de Dados - SysCall.xlsx
+++ b/SysCall-BackEnd/Dicionario de Dados/Dicionario de Dados - SysCall.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rsilva\Desktop\Syscall\SysCall-BackEnd\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rapha\Desktop\SysCall\SysCall-BackEnd\SysCall-BackEnd\Dicionario de Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D71290A8-B0B5-42D9-913D-D6675FD3AB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{13411CF3-6003-4221-8E7B-19D9DC3677E8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
     <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,12 +36,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Raphael Silva</author>
   </authors>
   <commentList>
-    <comment ref="F13" authorId="0" shapeId="0" xr:uid="{5554EA66-9843-4707-8A7A-61FD3B4EBD22}">
+    <comment ref="F13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -71,10 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="60">
-  <si>
-    <t>auth.users</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="60">
   <si>
     <t>CAMPOS</t>
   </si>
@@ -106,12 +102,6 @@
     <t>TRIGGERS</t>
   </si>
   <si>
-    <t>...</t>
-  </si>
-  <si>
-    <t>ACTIONS</t>
-  </si>
-  <si>
     <t>TIPO</t>
   </si>
   <si>
@@ -175,12 +165,6 @@
     <t>status</t>
   </si>
   <si>
-    <t>schema_auth_saved_user</t>
-  </si>
-  <si>
-    <t>schema_auth_owner_user</t>
-  </si>
-  <si>
     <t>CHAR(1)</t>
   </si>
   <si>
@@ -190,12 +174,6 @@
     <t>date</t>
   </si>
   <si>
-    <t>schema_auth_recived_user</t>
-  </si>
-  <si>
-    <t>schema_auth_requester_user</t>
-  </si>
-  <si>
     <t>TIMESTAMP</t>
   </si>
   <si>
@@ -250,14 +228,35 @@
     <t>-</t>
   </si>
   <si>
-    <t xml:space="preserve">tid </t>
+    <t>public.call_user</t>
+  </si>
+  <si>
+    <t>saved_user</t>
+  </si>
+  <si>
+    <t>owner_user</t>
+  </si>
+  <si>
+    <t>recived_user</t>
+  </si>
+  <si>
+    <t>requester_user</t>
+  </si>
+  <si>
+    <t>trg_insert_view_agenda</t>
+  </si>
+  <si>
+    <t>trg_update_view_agenda</t>
+  </si>
+  <si>
+    <t>trg_delete_view_agenda</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,6 +292,13 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -320,7 +326,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -613,11 +619,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -638,9 +659,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -715,6 +733,19 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1053,481 +1084,468 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2AACCDA-C29A-49F3-8E50-4F87A19374D8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:L49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="48.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="48.3984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="28" t="s">
+    <row r="3" spans="1:12" ht="14.4" thickBot="1"/>
+    <row r="4" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B4" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="29"/>
+      <c r="J4" s="36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B5" s="30"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="32"/>
+      <c r="J5" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="30"/>
-    </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="31"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="33"/>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="37" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="C7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="D7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="6" t="s">
+      <c r="E7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="J7" s="37" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="B8" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="H7" s="25" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H8" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15">
       <c r="A9" s="5"/>
       <c r="B9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15">
+      <c r="B10" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C10" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="15">
+      <c r="B11" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="15">
+      <c r="B12" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H9" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="12" t="s">
+      <c r="D12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15">
+      <c r="B13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H10" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="D13" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H11" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="12" t="s">
+      <c r="E13" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B14" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H12" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H13" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="F14" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="G14" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="8"/>
+      <c r="D14" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H14" s="26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="C15" s="33"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="1"/>
       <c r="H15" s="1"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="11"/>
+    </row>
+    <row r="16" spans="1:12">
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
-      <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="11"/>
+    <row r="17" spans="1:12">
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
     </row>
-    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="11"/>
+    <row r="18" spans="1:12">
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
     </row>
-    <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B23" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="30"/>
-    </row>
-    <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="31"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="33"/>
-    </row>
-    <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="14.4" thickBot="1"/>
+    <row r="23" spans="1:12">
+      <c r="B23" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="29"/>
+    </row>
+    <row r="24" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B24" s="30"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="32"/>
+    </row>
+    <row r="25" spans="1:12" ht="14.4" thickBot="1">
       <c r="B25" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="H25" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F25" s="2" t="s">
+    </row>
+    <row r="26" spans="1:12" ht="15">
+      <c r="B26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="D26" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H25" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="H26" s="25" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H27" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E26" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H26" s="24" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="15">
+      <c r="B27" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="15">
       <c r="A28" s="5"/>
       <c r="B28" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="H28" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B29" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C29" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="H28" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="B29" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H29" s="26" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="12" t="s">
+    </row>
+    <row r="30" spans="1:12" ht="14.4" thickBot="1">
+      <c r="B30" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H30" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="H30" s="27" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" s="8"/>
-      <c r="D31" s="7"/>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="B31" s="33"/>
+      <c r="D31" s="34"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="H31" s="7"/>
     </row>
-    <row r="32" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C32" s="11"/>
+    <row r="32" spans="1:12">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -1536,11 +1554,7 @@
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="11"/>
+    <row r="33" spans="2:12">
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -1551,11 +1565,7 @@
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
     </row>
-    <row r="34" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C34" s="11"/>
+    <row r="34" spans="2:12">
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -1566,185 +1576,172 @@
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="J36" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="37" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="28" t="s">
+    <row r="37" spans="2:12" ht="14.4" thickBot="1"/>
+    <row r="38" spans="2:12">
+      <c r="B38" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="29"/>
+    </row>
+    <row r="39" spans="2:12" ht="14.4" thickBot="1">
+      <c r="B39" s="30"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="31"/>
+      <c r="H39" s="32"/>
+    </row>
+    <row r="40" spans="2:12" ht="14.4" thickBot="1">
+      <c r="B40" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="30"/>
-    </row>
-    <row r="39" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="31"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="33"/>
-    </row>
-    <row r="40" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C40" s="4" t="s">
+      <c r="F40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="H40" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E40" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F40" s="2" t="s">
+    </row>
+    <row r="41" spans="2:12">
+      <c r="B41" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="D41" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H40" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B41" s="6" t="s">
+      <c r="E41" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H41" s="24" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12">
+      <c r="B42" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="D42" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G42" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H42" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="2:12">
+      <c r="B43" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H43" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="44" spans="2:12">
+      <c r="B44" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G44" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H44" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D41" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F41" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G41" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="H41" s="25" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B42" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D42" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E42" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="F42" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G42" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H42" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B43" s="18" t="s">
+    </row>
+    <row r="45" spans="2:12" ht="14.4" thickBot="1">
+      <c r="B45" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C45" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E45" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C43" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G43" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H43" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B44" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C44" s="12" t="s">
+      <c r="F45" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G45" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H45" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D44" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E44" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F44" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G44" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="H44" s="26" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C45" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F45" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="G45" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="H45" s="27" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B46" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="8"/>
+    </row>
+    <row r="46" spans="2:12">
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="1"/>
       <c r="H46" s="7"/>
     </row>
-    <row r="47" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C47" s="11"/>
+    <row r="47" spans="2:12">
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -1753,11 +1750,7 @@
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B48" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C48" s="11"/>
+    <row r="48" spans="2:12">
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -1768,11 +1761,7 @@
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
     </row>
-    <row r="49" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C49" s="11"/>
+    <row r="49" spans="4:12">
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -1795,60 +1784,60 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33B8EA0-846C-4A94-A7DE-C43EB2EB6172}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C2:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="3:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C4" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C5" s="20" t="s">
+    <row r="2" spans="3:4" ht="15.75" thickBot="1"/>
+    <row r="3" spans="3:4" ht="15.75" thickBot="1">
+      <c r="C3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4" ht="15">
+      <c r="C4" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" ht="15">
+      <c r="C5" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C6" s="20" t="s">
+    </row>
+    <row r="6" spans="3:4" ht="15">
+      <c r="C6" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" ht="15">
+      <c r="C7" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="19" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C7" s="20" t="s">
+      <c r="D7" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="19" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C8" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>54</v>
+    </row>
+    <row r="8" spans="3:4" ht="15">
+      <c r="C8" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1866,12 +1855,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BDF39B024F04A14486BA613BEA42AFF1" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="48c91588e4c96d3b87372e2739b705e1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="87289aac-3191-415d-94b6-004c2ae78a31" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0362d00d4c3829c3077b766beca3d16d" ns3:_="">
     <xsd:import namespace="87289aac-3191-415d-94b6-004c2ae78a31"/>
@@ -2015,6 +1998,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{318E7733-B127-4355-B93C-6EC54A543DCE}">
   <ds:schemaRefs>
@@ -2024,22 +2013,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12E806BA-4CE2-430B-BCC3-C1004ADA0620}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="87289aac-3191-415d-94b6-004c2ae78a31"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D2CE125-FEC1-4111-B9B7-3D153BF8148D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2055,4 +2028,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12E806BA-4CE2-430B-BCC3-C1004ADA0620}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="87289aac-3191-415d-94b6-004c2ae78a31"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>